<commit_message>
chore(bench): regenerate the release workbook so it records the conditions it was produced under
</commit_message>
<xml_diff>
--- a/bench/rounds-ab/release_r2/R2_FBF10847_v0.16.58_amplicon_MAME.xlsx
+++ b/bench/rounds-ab/release_r2/R2_FBF10847_v0.16.58_amplicon_MAME.xlsx
@@ -48278,7 +48278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -48303,7 +48303,11 @@
           <t>kuma_version</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr"/>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>0.16.58</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -48313,17 +48317,173 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>2026-09-13T08:34:49Z</t>
+          <t>2026-09-14T05:12:52Z</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
+          <t>reference_file</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>pTSN-PtIspS-idi(KanR)_corrected.reference.amplicon.fa</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>reference_length</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>1715</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>reference_sha256</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>cf143e11ae9ef717e9d282317745a40528d7e3947cfb10741dbf967f343d9f11</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>coding_window</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>16-1699</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>amplicon</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>ingest_mode</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>barcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>min_read_count</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>max_consensus_n_fraction</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>min_file_size_kb</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>many_cutoff</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>mixed_confident_depth_factor</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>mixed_confident_read_count</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>verdict_classes</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>PASS, AMBIGUOUS, MIXED, FRAMESHIFT, MANY, LOWDEPTH, NO_CALL, WRONG_AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
           <t>ngs_run_meta</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>(not found, no MinKNOW run folder detected)</t>
         </is>

</xml_diff>

<commit_message>
chore(bench): record the sequencing run in the release workbook the driver already knew
</commit_message>
<xml_diff>
--- a/bench/rounds-ab/release_r2/R2_FBF10847_v0.16.58_amplicon_MAME.xlsx
+++ b/bench/rounds-ab/release_r2/R2_FBF10847_v0.16.58_amplicon_MAME.xlsx
@@ -48278,7 +48278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -48317,7 +48317,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>2026-09-14T05:12:52Z</t>
+          <t>2026-09-14T08:03:56Z</t>
         </is>
       </c>
     </row>
@@ -48480,12 +48480,96 @@
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>ngs_run_meta</t>
+          <t>instrument</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>(not found, no MinKNOW run folder detected)</t>
+          <t>GXB05358</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>X4</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>flow_cell_id</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>FBF10847</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>sample_id</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>260212_KHM</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>kit</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>SQK-NBD114-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>started</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-12T22:31:24.495269+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>basecalling_enabled</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>raw_run_dir</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>/mnt/d/_workspace/020.admin/projects/060.nanopore_NGS/20260212_2227_X4_FBF10847_e7145f8e</t>
         </is>
       </c>
     </row>

</xml_diff>